<commit_message>
Add royal celebration gala page, dual QR table tent cards studio, and QR endpoints
</commit_message>
<xml_diff>
--- a/Wageni_Waliotumiwa_WhatsApp_Safi_2026_10_11.xlsx
+++ b/Wageni_Waliotumiwa_WhatsApp_Safi_2026_10_11.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Waliotumiwa (Imefika)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Waliokwama (Hawakupokea)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Muhtasari wa Takwimu" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Orodha Kamili ya Wageni" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Zilizofika (IMEFIKA)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Zilizokwama (HAIJAFIKA)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,44 +30,46 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000B2240"/>
-      <sz val="13"/>
+      <color rgb="00102A45"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00555555"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00137333"/>
-      <sz val="10"/>
+      <color rgb="001B2A3D"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00222222"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C5221F"/>
-      <sz val="13"/>
+      <color rgb="000D652D"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000B2240"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="10"/>
+      <color rgb="00B31412"/>
+      <sz val="15"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -76,8 +78,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000B2240"/>
-        <bgColor rgb="000B2240"/>
+        <fgColor rgb="00102A45"/>
+        <bgColor rgb="00102A45"/>
       </patternFill>
     </fill>
     <fill>
@@ -88,14 +90,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="008A1B14"/>
-        <bgColor rgb="008A1B14"/>
+        <fgColor rgb="00F9FAFB"/>
+        <bgColor rgb="00F9FAFB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CBA135"/>
-        <bgColor rgb="00CBA135"/>
+        <fgColor rgb="000D652D"/>
+        <bgColor rgb="000D652D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008A1B14"/>
+        <bgColor rgb="008A1B14"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,50 +117,69 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00CCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00CCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00CCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -518,152 +545,127 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="77" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ORODHA YA WAGENI WALIOTUMIWA KADI YA WHATSAPP (SEND-OFF YA LILIAN MARCUS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+          <t>ORODHA YA WAGENI WALIOTUMIWA UJUMBE WA WHATSAPP (SEND-OFF YA LILIAN MARCUS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Jumla ya Wageni: 2  |  ✅ Zilizofika (IMEFIKA): 2  |  ❌ Zilizokwama (HAIJAFIKA): 0  |  Tarehe: 11/10/2026 15:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Na.</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Jina la Mgeni</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Namba ya WhatsApp</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Viti</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Hali ya Utumaji</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Mtoa Huduma</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Namba ya Simu</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Aina ya Mwaliko</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Hali ya Ujumbe</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Muda Uliotumwa</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Maelezo ya Utumaji</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="3" t="n">
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Felician Joseph</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>+255787661560</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Double (2)</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>IMEFIKA</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>UltraMsg</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>2026-10-10 12:35</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Ilifanikiwa baada ya kurudiwa</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="n">
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Mr &amp; Mrs Bright Nyahende</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>+255756670798</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Double (2)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>IMEFIKA</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>UltraMsg</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>2026-10-09 09:24</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Ilifika mara ya kwanza</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -675,66 +677,119 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="67" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>ORODHA YA WAGENI WAMBAO UJUMBE WA WHATSAPP ULIKWAMA (HAUKUFIKA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>WAGENI WALIOFIKIWA KWA MAFANIKIO (Jumla: 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Na.</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Jina la Mgeni</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Namba ya WhatsApp</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Viti</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>Hali ya Utumaji</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Mtoa Huduma</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>Hatua Inayopendekezwa</t>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>Namba ya Simu</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Aina ya Mwaliko</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>Hali ya Ujumbe</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>Muda Uliotumwa</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Felician Joseph</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>+255787661560</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Double (2)</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>IMEFIKA</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-10 12:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Mr &amp; Mrs Bright Nyahende</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>+255756670798</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Double (2)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>IMEFIKA</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-09 09:24</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -746,103 +801,59 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
-        <is>
-          <t>RIPOTI NA MUHTASARI WA UTUMAJI WA KADI ZA WHATSAPP</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
-        <is>
-          <t>Kipengele / Maelezo</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Takwimu</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Asilimia (%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>Jumla ya Wageni wa Kipekee Waliojaribiwa</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>Waliopokea Kadi kwa Mafanikio (Delivered)</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>Waliokwama / Hawajapokea (Failed)</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>Tarehe ya Kuandaa Ripoti</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>11/10/2026 14:29</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>WAGENI WAMBAO UJUMBE HAUJAFIKA (Jumla: 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Na.</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>Jina la Mgeni</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Namba ya Simu</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>Aina ya Mwaliko</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>Hali ya Ujumbe</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>Muda Uliotumwa</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>